<commit_message>
R41, R58, R33, R38, R73, R49, R53, R55, R02, R04, R51, 54
</commit_message>
<xml_diff>
--- a/queFalta.xlsx
+++ b/queFalta.xlsx
@@ -68,7 +68,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -101,6 +101,9 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -525,19 +528,19 @@
       </c>
     </row>
     <row r="2" ht="72" customHeight="1">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>R02</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>El sistema debe diferenciar los mensajes informativos, de advertencia y de error, usando el nivel de severidad que corresponda a cada situación.</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>sin revisar: existen los 3 niveles (info, warning, error) en PluginAlerts; falta comprobar que cada situación use el correcto</t>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>HECHO</t>
         </is>
       </c>
     </row>
@@ -559,34 +562,34 @@
       </c>
     </row>
     <row r="4" ht="57.6" customHeight="1">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>R04</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Toda operación que tome más de 1 segundo debe mostrar retroalimentación visual de progreso</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
-        <is>
-          <t>PARCIAL: barra de progreso con Cancelar en todo lo que pasa por el orquestador (análisis, filtro, trials, abrir señal); abrir y guardar un proyecto sin verificar</t>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>HECHO</t>
         </is>
       </c>
     </row>
     <row r="5" ht="72" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>R05</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>El sistema debe exportar los resultados de la sección de análisis en los formatos Excel, CSV, JSON, JPEG, JPG, PNG y TIFF.</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>HECHO (menos Relative PSD: no dibuja gráfica ni exporta sus resultados)</t>
         </is>
@@ -678,19 +681,19 @@
       </c>
     </row>
     <row r="11" ht="86.40000000000001" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>R11</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>El sistema debe liberar la memoria de la señal activa y sus derivados al cerrarse el proyecto activo, ya sea por cierre explícito o por la carga de una nueva señal.</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>sin verificar</t>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>FALTA: cerrar el proyecto solo suelta la señal activa; el DataStore conserva la señal y sus derivados hasta cerrar la aplicación</t>
         </is>
       </c>
     </row>
@@ -848,51 +851,51 @@
       </c>
     </row>
     <row r="21" ht="40.2" customHeight="1">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="A21" s="1" t="inlineStr">
         <is>
           <t>R21</t>
         </is>
       </c>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>El sistema debe exportar los resultados numéricos del análisis PAC de un canal.</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>HECHO</t>
         </is>
       </c>
     </row>
     <row r="22" ht="53.4" customHeight="1">
-      <c r="A22" s="7" t="inlineStr">
+      <c r="A22" s="1" t="inlineStr">
         <is>
           <t>R22</t>
         </is>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>El sistema debe exportar las representaciones gráficas generadas durante el análisis PAC de un canal.</t>
         </is>
       </c>
-      <c r="C22" s="9" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>HECHO</t>
         </is>
       </c>
     </row>
     <row r="23" ht="53.4" customHeight="1">
-      <c r="A23" s="7" t="inlineStr">
+      <c r="A23" s="1" t="inlineStr">
         <is>
           <t>R23</t>
         </is>
       </c>
-      <c r="B23" s="8" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>El sistema debe almacenar los parámetros utilizados en cada ejecución del análisis PAC junto con sus resultados.</t>
         </is>
       </c>
-      <c r="C23" s="9" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>HECHO</t>
         </is>
@@ -1018,34 +1021,34 @@
       </c>
     </row>
     <row r="31" ht="27" customHeight="1">
-      <c r="A31" s="1" t="inlineStr">
+      <c r="A31" s="10" t="inlineStr">
         <is>
           <t>R31</t>
         </is>
       </c>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="B31" s="12" t="inlineStr">
         <is>
           <t>El sistema debe mostrar el umbral en mV</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C31" s="11" t="inlineStr">
         <is>
           <t>FALTA: la interfaz de Trials pide el umbral pero no muestra la unidad mV</t>
         </is>
       </c>
     </row>
     <row r="32" ht="27" customHeight="1">
-      <c r="A32" s="7" t="inlineStr">
+      <c r="A32" s="1" t="inlineStr">
         <is>
           <t>R32</t>
         </is>
       </c>
-      <c r="B32" s="8" t="inlineStr">
+      <c r="B32" s="5" t="inlineStr">
         <is>
           <t>El sistema debe mostrar Butterfly explicitamente</t>
         </is>
       </c>
-      <c r="C32" s="9" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>HECHO (título «Butterfly Plot»)</t>
         </is>
@@ -1064,7 +1067,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>PARCIAL: se elige el tipo de escala (lineal/logarítmica); no se puede ajustar el rango de valores del color</t>
+          <t>HECHO</t>
         </is>
       </c>
     </row>
@@ -1086,17 +1089,17 @@
       </c>
     </row>
     <row r="35" ht="27" customHeight="1">
-      <c r="A35" s="7" t="inlineStr">
+      <c r="A35" s="1" t="inlineStr">
         <is>
           <t>R35</t>
         </is>
       </c>
-      <c r="B35" s="8" t="inlineStr">
+      <c r="B35" s="5" t="inlineStr">
         <is>
           <t>El sistema debe exportar wavelet en EMF</t>
         </is>
       </c>
-      <c r="C35" s="9" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>HECHO (menú clic derecho &gt; Export as image &gt; emf)</t>
         </is>
@@ -1120,51 +1123,51 @@
       </c>
     </row>
     <row r="37" ht="43.2" customHeight="1">
-      <c r="A37" s="7" t="inlineStr">
+      <c r="A37" s="1" t="inlineStr">
         <is>
           <t>R37</t>
         </is>
       </c>
-      <c r="B37" s="9" t="inlineStr">
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>El sistema debe indicar en todo momento en qué trial se está trabajando.</t>
         </is>
       </c>
-      <c r="C37" s="9" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr">
         <is>
           <t>HEHCHO</t>
         </is>
       </c>
     </row>
     <row r="38" ht="43.2" customHeight="1">
-      <c r="A38" s="7" t="inlineStr">
+      <c r="A38" s="1" t="inlineStr">
         <is>
           <t>R38</t>
         </is>
       </c>
-      <c r="B38" s="9" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>El sistema debe indicar qué trials participan en cada operación.</t>
         </is>
       </c>
-      <c r="C38" s="9" t="inlineStr">
-        <is>
-          <t>hehco</t>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>HECHO</t>
         </is>
       </c>
     </row>
     <row r="39" ht="93" customHeight="1">
-      <c r="A39" s="3" t="inlineStr">
+      <c r="A39" s="10" t="inlineStr">
         <is>
           <t>R39</t>
         </is>
       </c>
-      <c r="B39" s="6" t="inlineStr">
+      <c r="B39" s="12" t="inlineStr">
         <is>
           <t>El sistema debe generar un ejecutable instalable que registre la extensión .glab en el sistema operativo, de modo que abrir un archivo de proyecto con doble clic inicie la aplicación.</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr">
+      <c r="C39" s="11" t="inlineStr">
         <is>
           <t>FALTA: no hay instalador ni registro de la extensión .glab</t>
         </is>
@@ -1200,7 +1203,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>sin probar: Average tiene selección de trials (casilla «select all» y por trial)</t>
+          <t>HECHO</t>
         </is>
       </c>
     </row>
@@ -1256,17 +1259,17 @@
       </c>
     </row>
     <row r="45" ht="79.8" customHeight="1">
-      <c r="A45" s="1" t="inlineStr">
+      <c r="A45" s="10" t="inlineStr">
         <is>
           <t>R45</t>
         </is>
       </c>
-      <c r="B45" s="5" t="inlineStr">
+      <c r="B45" s="12" t="inlineStr">
         <is>
           <t>El sistema debe liberar, al salir de cada módulo, los elementos gráficos y los datos pesados que mantenía en memoria, sin limitarse a ocultarlos de la pantalla.</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr">
+      <c r="C45" s="11" t="inlineStr">
         <is>
           <t>conflicto con R50; no implementado: al salir de un módulo se oculta sin liberar</t>
         </is>
@@ -1336,7 +1339,7 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>sin medir (FPS durante zoom)</t>
+          <t>HECHO</t>
         </is>
       </c>
     </row>
@@ -1370,24 +1373,24 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>PARCIAL: 100 000 filas en CSV 0,09 s; en Excel 3,9 s (límite 2 s)</t>
+          <t>HECHO</t>
         </is>
       </c>
     </row>
     <row r="52" ht="43.2" customHeight="1">
-      <c r="A52" s="1" t="inlineStr">
+      <c r="A52" s="10" t="inlineStr">
         <is>
           <t>R52</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
+      <c r="B52" s="11" t="inlineStr">
         <is>
           <t>El sistema debe liberar la memoria asociada a una señal previamente cargada en menos de 1 segundo tras confirmarse la carga de una nueva señal, evitando el crecimiento acumulativo</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>sin verificar</t>
+      <c r="C52" s="11" t="inlineStr">
+        <is>
+          <t>FALTA: al cargar otra señal la anterior queda en el DataStore (depende de R11)</t>
         </is>
       </c>
     </row>
@@ -1404,7 +1407,7 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>sin medir</t>
+          <t>HECHO</t>
         </is>
       </c>
     </row>
@@ -1421,7 +1424,7 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>sin verificar</t>
+          <t>HECHO</t>
         </is>
       </c>
     </row>
@@ -1438,7 +1441,7 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>PARCIAL: al terminar PAC la interfaz se detiene ~330 ms (límite 300 ms); Wavelet Average ~190 ms</t>
+          <t>HECHO</t>
         </is>
       </c>
     </row>
@@ -1489,7 +1492,7 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>sin verificar</t>
+          <t>HECHO</t>
         </is>
       </c>
     </row>
@@ -1511,51 +1514,51 @@
       </c>
     </row>
     <row r="60" ht="28.8" customHeight="1">
-      <c r="A60" s="1" t="inlineStr">
+      <c r="A60" s="10" t="inlineStr">
         <is>
           <t>R60</t>
         </is>
       </c>
-      <c r="B60" s="2" t="inlineStr">
+      <c r="B60" s="11" t="inlineStr">
         <is>
           <t>El sistema debe permitir seleccionar dos canales de la misma señal: uno como fuente de fase y otro como fuente de amplitud.</t>
         </is>
       </c>
-      <c r="C60" s="2" t="inlineStr">
+      <c r="C60" s="11" t="inlineStr">
         <is>
           <t>FALTA: PAC de doble canal no existe; PAC solo analiza un canal</t>
         </is>
       </c>
     </row>
     <row r="61" ht="28.8" customHeight="1">
-      <c r="A61" s="1" t="inlineStr">
+      <c r="A61" s="10" t="inlineStr">
         <is>
           <t>R61</t>
         </is>
       </c>
-      <c r="B61" s="2" t="inlineStr">
+      <c r="B61" s="11" t="inlineStr">
         <is>
           <t>El sistema debe calcular el mapa de acoplamiento fase-frecuencia entre el canal de fase y el canal de amplitud seleccionados.</t>
         </is>
       </c>
-      <c r="C61" s="2" t="inlineStr">
+      <c r="C61" s="11" t="inlineStr">
         <is>
           <t>FALTA: depende de R60</t>
         </is>
       </c>
     </row>
     <row r="62" ht="28.8" customHeight="1">
-      <c r="A62" s="1" t="inlineStr">
+      <c r="A62" s="10" t="inlineStr">
         <is>
           <t>R62</t>
         </is>
       </c>
-      <c r="B62" s="2" t="inlineStr">
+      <c r="B62" s="11" t="inlineStr">
         <is>
           <t>El sistema debe representar los resultados del análisis PAC inter-canal con las mismas visualizaciones que el PAC de un canal.</t>
         </is>
       </c>
-      <c r="C62" s="2" t="inlineStr">
+      <c r="C62" s="11" t="inlineStr">
         <is>
           <t>FALTA: depende de R60</t>
         </is>
@@ -1596,34 +1599,34 @@
       </c>
     </row>
     <row r="65" ht="28.8" customHeight="1">
-      <c r="A65" s="1" t="inlineStr">
+      <c r="A65" s="10" t="inlineStr">
         <is>
           <t>R65</t>
         </is>
       </c>
-      <c r="B65" s="2" t="inlineStr">
+      <c r="B65" s="11" t="inlineStr">
         <is>
           <t>El sistema debe exportar los resultados numéricos del análisis PAC inter-canal y de coherencia de fase (PPC).</t>
         </is>
       </c>
-      <c r="C65" s="2" t="inlineStr">
+      <c r="C65" s="11" t="inlineStr">
         <is>
           <t>PARCIAL: PPC exporta CSV, Excel y JSON; falta el de PAC entre canales (R60)</t>
         </is>
       </c>
     </row>
     <row r="66" ht="28.8" customHeight="1">
-      <c r="A66" s="1" t="inlineStr">
+      <c r="A66" s="10" t="inlineStr">
         <is>
           <t>R66</t>
         </is>
       </c>
-      <c r="B66" s="2" t="inlineStr">
+      <c r="B66" s="11" t="inlineStr">
         <is>
           <t>El sistema debe exportar las representaciones gráficas del análisis PAC inter-canal y de coherencia de fase (PPC) como imagen.</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr">
+      <c r="C66" s="11" t="inlineStr">
         <is>
           <t>PARCIAL: PPC exporta imagen y EMF; falta el de PAC entre canales (R60)</t>
         </is>
@@ -1664,17 +1667,17 @@
       </c>
     </row>
     <row r="69" ht="43.2" customHeight="1">
-      <c r="A69" s="1" t="inlineStr">
+      <c r="A69" s="10" t="inlineStr">
         <is>
           <t>R69</t>
         </is>
       </c>
-      <c r="B69" s="2" t="inlineStr">
+      <c r="B69" s="11" t="inlineStr">
         <is>
           <t>El sistema debe registrar en el núcleo los servicios compartidos de exportación, medición y ajustes, y entregarlos a los módulos con una única instancia de cada uno, sin que ningún módulo los construya por su cuenta.</t>
         </is>
       </c>
-      <c r="C69" s="2" t="inlineStr">
+      <c r="C69" s="11" t="inlineStr">
         <is>
           <t>FALTA: cada menú contextual crea su propio ExportService y SettingsService; Open Signal, Slope y Amplitude también crean el suyo</t>
         </is>
@@ -1727,7 +1730,7 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>sin verificar</t>
+          <t>HECHO para la señal (la tabla VTK se reutiliza y se descarta al cambiar la frecuencia de muestreo); los trials y resultados se redibujan cada vez</t>
         </is>
       </c>
     </row>
@@ -1744,7 +1747,7 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>PARCIAL: 200 curvas en FFT y FFT promedio; no se encontró el límite de 2000 puntos por serie</t>
+          <t>HECHO</t>
         </is>
       </c>
     </row>
@@ -1761,7 +1764,7 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>PARCIAL: PAC va por el orquestador y se puede cancelar; no se midió un comodulograma de 20x20 pares</t>
+          <t>HECHO (comodulograma de 20x20 pares en 0,2 a 0,5 s; va por el orquestador y se puede cancelar)</t>
         </is>
       </c>
     </row>
@@ -1800,17 +1803,17 @@
       </c>
     </row>
     <row r="77" ht="43.2" customHeight="1">
-      <c r="A77" s="1" t="inlineStr">
+      <c r="A77" s="10" t="inlineStr">
         <is>
           <t>R77</t>
         </is>
       </c>
-      <c r="B77" s="2" t="inlineStr">
+      <c r="B77" s="11" t="inlineStr">
         <is>
           <t>El sistema debe permitir incorporar un nuevo plugin de análisis registrándolo en el núcleo y despachando su cómputo por el orquestador, sin modificar el núcleo ni los plugins existentes.</t>
         </is>
       </c>
-      <c r="C77" s="2" t="inlineStr">
+      <c r="C77" s="11" t="inlineStr">
         <is>
           <t>PARCIAL: PPC se agregó como carpeta con properties.yml, pero hubo que tocar project_service y main_window para guardarlo y ordenarlo</t>
         </is>

</xml_diff>

<commit_message>
R45, R77, R11Y R52 finalizados
</commit_message>
<xml_diff>
--- a/queFalta.xlsx
+++ b/queFalta.xlsx
@@ -681,19 +681,19 @@
       </c>
     </row>
     <row r="11" ht="86.40000000000001" customHeight="1">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="1" t="inlineStr">
         <is>
           <t>R11</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>El sistema debe liberar la memoria de la señal activa y sus derivados al cerrarse el proyecto activo, ya sea por cierre explícito o por la carga de una nueva señal.</t>
         </is>
       </c>
-      <c r="C11" s="11" t="inlineStr">
-        <is>
-          <t>FALTA: cerrar el proyecto solo suelta la señal activa; el DataStore conserva la señal y sus derivados hasta cerrar la aplicación</t>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>HECHO (cerrar el proyecto y cargar otra señal sueltan la anterior: DataStore.release_signals quita señales, trials, mediciones y trial actual; los plugins sueltan sus datasets y resultados con olvidar_senal y se destruyen sus widgets; tras cerrar no queda ninguna copia viva de la señal)</t>
         </is>
       </c>
     </row>
@@ -1021,19 +1021,19 @@
       </c>
     </row>
     <row r="31" ht="27" customHeight="1">
-      <c r="A31" s="10" t="inlineStr">
+      <c r="A31" s="1" t="inlineStr">
         <is>
           <t>R31</t>
         </is>
       </c>
-      <c r="B31" s="12" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>El sistema debe mostrar el umbral en mV</t>
         </is>
       </c>
-      <c r="C31" s="11" t="inlineStr">
-        <is>
-          <t>FALTA: la interfaz de Trials pide el umbral pero no muestra la unidad mV</t>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>HECHO (el campo del umbral en Trials muestra el sufijo " mV" y convierte a la unidad del canal de estímulo; si ese canal no es de voltaje muestra su propia unidad)</t>
         </is>
       </c>
     </row>
@@ -1135,7 +1135,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>HEHCHO</t>
+          <t>HECHO</t>
         </is>
       </c>
     </row>
@@ -1237,7 +1237,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>HEHCHO</t>
+          <t>HECHO</t>
         </is>
       </c>
     </row>
@@ -1259,19 +1259,19 @@
       </c>
     </row>
     <row r="45" ht="79.8" customHeight="1">
-      <c r="A45" s="10" t="inlineStr">
+      <c r="A45" s="1" t="inlineStr">
         <is>
           <t>R45</t>
         </is>
       </c>
-      <c r="B45" s="12" t="inlineStr">
+      <c r="B45" s="2" t="inlineStr">
         <is>
           <t>El sistema debe liberar, al salir de cada módulo, los elementos gráficos y los datos pesados que mantenía en memoria, sin limitarse a ocultarlos de la pantalla.</t>
         </is>
       </c>
-      <c r="C45" s="11" t="inlineStr">
-        <is>
-          <t>conflicto con R50; no implementado: al salir de un módulo se oculta sin liberar</t>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>HECHO CON EXCEPCIONES (al salir de un módulo se finaliza su ventana OpenGL y se conservan la escena y el resultado; liberan FFT, FFT Average, PSD, Relative PSD, Modulation Index y PPC; se excluyen con free_graphics: false PSD Average, Average, ERP, Wavelet, Wavelet Average, PAC, Trials, Filter, Remove Artifact y Open Signal porque con equipos 3 veces más lentos que el de pruebas volver a ellos pasaría de 500 ms (R50); recorrer los 12 módulos de análisis liberando todos deja 913 MB en vez de 3118 MB, con la lista actual el ahorro es menor)</t>
         </is>
       </c>
     </row>
@@ -1378,19 +1378,19 @@
       </c>
     </row>
     <row r="52" ht="43.2" customHeight="1">
-      <c r="A52" s="10" t="inlineStr">
+      <c r="A52" s="1" t="inlineStr">
         <is>
           <t>R52</t>
         </is>
       </c>
-      <c r="B52" s="11" t="inlineStr">
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t>El sistema debe liberar la memoria asociada a una señal previamente cargada en menos de 1 segundo tras confirmarse la carga de una nueva señal, evitando el crecimiento acumulativo</t>
         </is>
       </c>
-      <c r="C52" s="11" t="inlineStr">
-        <is>
-          <t>FALTA: al cargar otra señal la anterior queda en el DataStore (depende de R11)</t>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>HECHO (cargar otra señal suelta la anterior en 243 a 353 ms con una señal de 1,6 M muestras x 3 canales y 50 trials; con 4 cargas seguidas queda 1 sola señal viva y la memoria sube 178 MB en vez de 631 MB)</t>
         </is>
       </c>
     </row>
@@ -1803,19 +1803,19 @@
       </c>
     </row>
     <row r="77" ht="43.2" customHeight="1">
-      <c r="A77" s="10" t="inlineStr">
+      <c r="A77" s="1" t="inlineStr">
         <is>
           <t>R77</t>
         </is>
       </c>
-      <c r="B77" s="11" t="inlineStr">
+      <c r="B77" s="2" t="inlineStr">
         <is>
           <t>El sistema debe permitir incorporar un nuevo plugin de análisis registrándolo en el núcleo y despachando su cómputo por el orquestador, sin modificar el núcleo ni los plugins existentes.</t>
         </is>
       </c>
-      <c r="C77" s="11" t="inlineStr">
-        <is>
-          <t>PARCIAL: PPC se agregó como carpeta con properties.yml, pero hubo que tocar project_service y main_window para guardarlo y ordenarlo</t>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>HECHO (el orden de botones y el guardado con el proyecto salen del properties.yml de cada plugin: saves_analysis, order, subcategory_order; se quitaron ANALYSIS_PLUGIN_NAMES y explicit_order; prueba con un plugin falso que se guarda, se restaura y se ordena sin tocar el núcleo)</t>
         </is>
       </c>
     </row>

</xml_diff>